<commit_message>
Update Excel data files and gitignore
</commit_message>
<xml_diff>
--- a/data/premier_league_raw_match_data.xlsx
+++ b/data/premier_league_raw_match_data.xlsx
@@ -5,22 +5,23 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Daniel\Downloads\Nowy folder\112\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Daniel\Desktop\InStatsWeTrust\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B136C811-3BB4-470B-8DFE-0971E06846D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9347771-FD1F-4E20-9650-21526F05ED8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27210" yWindow="3360" windowWidth="25875" windowHeight="13455" xr2:uid="{0FE85BFC-2024-4027-B3AD-B7D6B58B61DA}"/>
+    <workbookView xWindow="-28245" yWindow="2325" windowWidth="25875" windowHeight="13455" xr2:uid="{0FE85BFC-2024-4027-B3AD-B7D6B58B61DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1659" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1776" uniqueCount="102">
   <si>
     <t>Manchester City</t>
   </si>
@@ -273,6 +274,60 @@
   <si>
     <t>Round</t>
   </si>
+  <si>
+    <t>Etihad Stadium</t>
+  </si>
+  <si>
+    <t>Craig Pawson</t>
+  </si>
+  <si>
+    <t>Match Report</t>
+  </si>
+  <si>
+    <t>Emirates Stadium</t>
+  </si>
+  <si>
+    <t>Michael Salisbury</t>
+  </si>
+  <si>
+    <t>Stamford Bridge</t>
+  </si>
+  <si>
+    <t>Chris Kavanagh</t>
+  </si>
+  <si>
+    <t>The American Express Stadium</t>
+  </si>
+  <si>
+    <t>Darren England</t>
+  </si>
+  <si>
+    <t>Molineux Stadium</t>
+  </si>
+  <si>
+    <t>Samuel Barrott</t>
+  </si>
+  <si>
+    <t>St Mary's Stadium</t>
+  </si>
+  <si>
+    <t>Tony Harrington</t>
+  </si>
+  <si>
+    <t>St James' Park</t>
+  </si>
+  <si>
+    <t>Vitality Stadium</t>
+  </si>
+  <si>
+    <t>Peter Bankes</t>
+  </si>
+  <si>
+    <t>Anfield</t>
+  </si>
+  <si>
+    <t>Thomas Bramall</t>
+  </si>
 </sst>
 </file>
 
@@ -306,9 +361,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -643,7 +699,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A647DF9E-0117-4165-BE47-DD1C6849A118}">
-  <dimension ref="A1:I331"/>
+  <dimension ref="A1:J340"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
@@ -9935,7 +9991,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="321" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A321">
         <v>29</v>
       </c>
@@ -9964,7 +10020,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="322" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A322">
         <v>33</v>
       </c>
@@ -9993,7 +10049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="323" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A323">
         <v>33</v>
       </c>
@@ -10022,7 +10078,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="324" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A324">
         <v>33</v>
       </c>
@@ -10051,7 +10107,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="325" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A325">
         <v>33</v>
       </c>
@@ -10080,7 +10136,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="326" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A326">
         <v>33</v>
       </c>
@@ -10109,7 +10165,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="327" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A327">
         <v>33</v>
       </c>
@@ -10138,7 +10194,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="328" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A328">
         <v>33</v>
       </c>
@@ -10167,7 +10223,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="329" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A329">
         <v>33</v>
       </c>
@@ -10196,7 +10252,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="330" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A330">
         <v>33</v>
       </c>
@@ -10225,7 +10281,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="331" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A331">
         <v>33</v>
       </c>
@@ -10253,9 +10309,658 @@
       <c r="I331" t="s">
         <v>21</v>
       </c>
+    </row>
+    <row r="332" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A332">
+        <v>34</v>
+      </c>
+      <c r="B332" t="s">
+        <v>64</v>
+      </c>
+      <c r="C332" s="1">
+        <v>45769</v>
+      </c>
+      <c r="D332" t="s">
+        <v>6</v>
+      </c>
+      <c r="E332" t="s">
+        <v>0</v>
+      </c>
+      <c r="F332">
+        <v>1.3</v>
+      </c>
+      <c r="G332" t="s">
+        <v>32</v>
+      </c>
+      <c r="H332">
+        <v>1.8</v>
+      </c>
+      <c r="I332" t="s">
+        <v>1</v>
+      </c>
+      <c r="J332" s="2"/>
+    </row>
+    <row r="333" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A333">
+        <v>34</v>
+      </c>
+      <c r="B333" t="s">
+        <v>67</v>
+      </c>
+      <c r="C333" s="1">
+        <v>45770</v>
+      </c>
+      <c r="D333" t="s">
+        <v>6</v>
+      </c>
+      <c r="E333" t="s">
+        <v>2</v>
+      </c>
+      <c r="F333">
+        <v>1.2</v>
+      </c>
+      <c r="G333" t="s">
+        <v>53</v>
+      </c>
+      <c r="H333">
+        <v>1.7</v>
+      </c>
+      <c r="I333" t="s">
+        <v>33</v>
+      </c>
+      <c r="J333" s="2"/>
+    </row>
+    <row r="334" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A334">
+        <v>34</v>
+      </c>
+      <c r="B334" t="s">
+        <v>10</v>
+      </c>
+      <c r="C334" s="1">
+        <v>45773</v>
+      </c>
+      <c r="D334" t="s">
+        <v>11</v>
+      </c>
+      <c r="E334" t="s">
+        <v>35</v>
+      </c>
+      <c r="F334">
+        <v>0.8</v>
+      </c>
+      <c r="G334" t="s">
+        <v>8</v>
+      </c>
+      <c r="H334">
+        <v>0.4</v>
+      </c>
+      <c r="I334" t="s">
+        <v>18</v>
+      </c>
+      <c r="J334" s="2"/>
+    </row>
+    <row r="335" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A335">
+        <v>34</v>
+      </c>
+      <c r="B335" t="s">
+        <v>10</v>
+      </c>
+      <c r="C335" s="1">
+        <v>45773</v>
+      </c>
+      <c r="D335" t="s">
+        <v>15</v>
+      </c>
+      <c r="E335" t="s">
+        <v>20</v>
+      </c>
+      <c r="F335">
+        <v>1.3</v>
+      </c>
+      <c r="G335" t="s">
+        <v>55</v>
+      </c>
+      <c r="H335">
+        <v>1.3</v>
+      </c>
+      <c r="I335" t="s">
+        <v>27</v>
+      </c>
+      <c r="J335" s="2"/>
+    </row>
+    <row r="336" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A336">
+        <v>34</v>
+      </c>
+      <c r="B336" t="s">
+        <v>10</v>
+      </c>
+      <c r="C336" s="1">
+        <v>45773</v>
+      </c>
+      <c r="D336" t="s">
+        <v>15</v>
+      </c>
+      <c r="E336" t="s">
+        <v>25</v>
+      </c>
+      <c r="F336">
+        <v>2</v>
+      </c>
+      <c r="G336" t="s">
+        <v>56</v>
+      </c>
+      <c r="H336">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="I336" t="s">
+        <v>37</v>
+      </c>
+      <c r="J336" s="2"/>
+    </row>
+    <row r="337" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A337">
+        <v>34</v>
+      </c>
+      <c r="B337" t="s">
+        <v>10</v>
+      </c>
+      <c r="C337" s="1">
+        <v>45773</v>
+      </c>
+      <c r="D337" t="s">
+        <v>15</v>
+      </c>
+      <c r="E337" t="s">
+        <v>17</v>
+      </c>
+      <c r="F337">
+        <v>0.6</v>
+      </c>
+      <c r="G337" t="s">
+        <v>28</v>
+      </c>
+      <c r="H337">
+        <v>2.4</v>
+      </c>
+      <c r="I337" t="s">
+        <v>9</v>
+      </c>
+      <c r="J337" s="2"/>
+    </row>
+    <row r="338" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A338">
+        <v>34</v>
+      </c>
+      <c r="B338" t="s">
+        <v>10</v>
+      </c>
+      <c r="C338" s="1">
+        <v>45773</v>
+      </c>
+      <c r="D338" t="s">
+        <v>15</v>
+      </c>
+      <c r="E338" t="s">
+        <v>16</v>
+      </c>
+      <c r="F338">
+        <v>2.4</v>
+      </c>
+      <c r="G338" t="s">
+        <v>56</v>
+      </c>
+      <c r="H338">
+        <v>0.1</v>
+      </c>
+      <c r="I338" t="s">
+        <v>12</v>
+      </c>
+      <c r="J338" s="2"/>
+    </row>
+    <row r="339" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A339">
+        <v>34</v>
+      </c>
+      <c r="B339" t="s">
+        <v>29</v>
+      </c>
+      <c r="C339" s="1">
+        <v>45774</v>
+      </c>
+      <c r="D339" t="s">
+        <v>30</v>
+      </c>
+      <c r="E339" t="s">
+        <v>23</v>
+      </c>
+      <c r="F339">
+        <v>0.5</v>
+      </c>
+      <c r="G339" t="s">
+        <v>22</v>
+      </c>
+      <c r="H339">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="I339" t="s">
+        <v>7</v>
+      </c>
+      <c r="J339" s="2"/>
+    </row>
+    <row r="340" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A340">
+        <v>34</v>
+      </c>
+      <c r="B340" t="s">
+        <v>29</v>
+      </c>
+      <c r="C340" s="1">
+        <v>45774</v>
+      </c>
+      <c r="D340" t="s">
+        <v>34</v>
+      </c>
+      <c r="E340" t="s">
+        <v>14</v>
+      </c>
+      <c r="F340">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="G340" t="s">
+        <v>81</v>
+      </c>
+      <c r="H340">
+        <v>0.5</v>
+      </c>
+      <c r="I340" t="s">
+        <v>38</v>
+      </c>
+      <c r="J340" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75" bottom="0.75" header="0.30000000000000004" footer="0.30000000000000004"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F15253A6-5A08-48CB-B2F0-10236C66CD3C}">
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <v>34</v>
+      </c>
+      <c r="B1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="1">
+        <v>45769</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1">
+        <v>1.3</v>
+      </c>
+      <c r="G1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1">
+        <v>1.8</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" s="2">
+        <v>51834</v>
+      </c>
+      <c r="K1" t="s">
+        <v>84</v>
+      </c>
+      <c r="L1" t="s">
+        <v>85</v>
+      </c>
+      <c r="M1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>34</v>
+      </c>
+      <c r="B2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" s="1">
+        <v>45770</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>1.2</v>
+      </c>
+      <c r="G2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H2">
+        <v>1.7</v>
+      </c>
+      <c r="I2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" s="2">
+        <v>60167</v>
+      </c>
+      <c r="K2" t="s">
+        <v>87</v>
+      </c>
+      <c r="L2" t="s">
+        <v>88</v>
+      </c>
+      <c r="M2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>34</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="1">
+        <v>45773</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3">
+        <v>0.8</v>
+      </c>
+      <c r="G3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3">
+        <v>0.4</v>
+      </c>
+      <c r="I3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" s="2">
+        <v>39894</v>
+      </c>
+      <c r="K3" t="s">
+        <v>89</v>
+      </c>
+      <c r="L3" t="s">
+        <v>90</v>
+      </c>
+      <c r="M3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>34</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="1">
+        <v>45773</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4">
+        <v>1.3</v>
+      </c>
+      <c r="G4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H4">
+        <v>1.3</v>
+      </c>
+      <c r="I4" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" s="2">
+        <v>31499</v>
+      </c>
+      <c r="K4" t="s">
+        <v>91</v>
+      </c>
+      <c r="L4" t="s">
+        <v>92</v>
+      </c>
+      <c r="M4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>34</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1">
+        <v>45773</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5" t="s">
+        <v>56</v>
+      </c>
+      <c r="H5">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="I5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J5" s="2">
+        <v>31518</v>
+      </c>
+      <c r="K5" t="s">
+        <v>93</v>
+      </c>
+      <c r="L5" t="s">
+        <v>94</v>
+      </c>
+      <c r="M5" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>34</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="1">
+        <v>45773</v>
+      </c>
+      <c r="D6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6">
+        <v>0.6</v>
+      </c>
+      <c r="G6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6">
+        <v>2.4</v>
+      </c>
+      <c r="I6" t="s">
+        <v>9</v>
+      </c>
+      <c r="J6" s="2">
+        <v>28946</v>
+      </c>
+      <c r="K6" t="s">
+        <v>95</v>
+      </c>
+      <c r="L6" t="s">
+        <v>96</v>
+      </c>
+      <c r="M6" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>34</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="1">
+        <v>45773</v>
+      </c>
+      <c r="D7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7">
+        <v>2.4</v>
+      </c>
+      <c r="G7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H7">
+        <v>0.1</v>
+      </c>
+      <c r="I7" t="s">
+        <v>12</v>
+      </c>
+      <c r="J7" s="2">
+        <v>52171</v>
+      </c>
+      <c r="K7" t="s">
+        <v>97</v>
+      </c>
+      <c r="L7" t="s">
+        <v>88</v>
+      </c>
+      <c r="M7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>34</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="1">
+        <v>45774</v>
+      </c>
+      <c r="D8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8">
+        <v>0.5</v>
+      </c>
+      <c r="G8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="I8" t="s">
+        <v>7</v>
+      </c>
+      <c r="J8" s="2">
+        <v>11241</v>
+      </c>
+      <c r="K8" t="s">
+        <v>98</v>
+      </c>
+      <c r="L8" t="s">
+        <v>99</v>
+      </c>
+      <c r="M8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>34</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="1">
+        <v>45774</v>
+      </c>
+      <c r="D9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="G9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H9">
+        <v>0.5</v>
+      </c>
+      <c r="I9" t="s">
+        <v>38</v>
+      </c>
+      <c r="J9" s="2">
+        <v>60415</v>
+      </c>
+      <c r="K9" t="s">
+        <v>100</v>
+      </c>
+      <c r="L9" t="s">
+        <v>101</v>
+      </c>
+      <c r="M9" t="s">
+        <v>86</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>